<commit_message>
Add target price margin calculator sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/PLC_견적_요약.xlsx
+++ b/PLC_견적_요약.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="요약" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="단가표" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="CPU 할인 효과" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="프로젝트별 구성" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="마진 계산" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="단가표" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="CPU 할인 효과" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="프로젝트별 구성" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="132">
   <si>
     <r>
       <rPr>
@@ -1267,6 +1268,716 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">타겟 프라이스 → 우리 마진</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">노란 칸</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 프라이스 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고객에게 파는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대 가격</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 금액을 넣으면 마진이 바로 계산됩니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) TSU DC24V </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">칸에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">450,000 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">입력</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">마진 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 프라이스 − 매입가     마진율 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">마진 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">÷ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 프라이스 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">판매가 기준</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">전원</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 수량
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매입가
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 프라이스
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">마진
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">마진율</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연간 매출</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연간 마진</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DC24V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">← 마진이 마이너스면 빨간색</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC220V</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 합계 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(4</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 프로젝트 전부</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">납품 방식</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연간 매입</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DC24V</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 납품</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AC220V</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 납품 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(MCC</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DC24V)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※ 연간 합계는 해당 납품 방식의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 칸을 모두 입력해야 나옵니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프로젝트별 마진은 위 표에서 바로 확인하세요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※ 매입가는 현재 할인율</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(CPU 0.45 / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확장 모듈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.40) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기준입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버스 확장 부품은 매입가에 포함되어 있지 않습니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF7F7F7F"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -1376,9 +2087,6 @@
     <t xml:space="preserve">모델</t>
   </si>
   <si>
-    <t xml:space="preserve">전원</t>
-  </si>
-  <si>
     <t xml:space="preserve">설명</t>
   </si>
   <si>
@@ -2251,51 +2959,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">연간 수량
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">대</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">연간 절감</t>
   </si>
   <si>
@@ -2771,9 +3434,6 @@
       </rPr>
       <t xml:space="preserve">대 가격</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">AC220V</t>
   </si>
   <si>
     <r>
@@ -3616,12 +4276,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\-#,##0;\-"/>
-    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3829,10 +4490,32 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1F3864"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF1F3864"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF1F3864"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -3854,14 +4537,6 @@
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
-      <name val="맑은 고딕"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF1F3864"/>
       <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
@@ -3925,7 +4600,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -3945,6 +4620,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
       </bottom>
       <diagonal/>
     </border>
@@ -3987,7 +4677,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="60">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4084,12 +4774,80 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -4100,7 +4858,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4108,7 +4866,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4116,39 +4874,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4160,15 +4906,15 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4181,6 +4927,17 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="맑은 고딕"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -4198,7 +4955,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
@@ -4230,7 +4987,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF595959"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -4424,7 +5181,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -4690,8 +5447,20 @@
       <c r="F20" s="23"/>
       <c r="G20" s="23"/>
     </row>
+    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="str">
+        <f aca="false">"⑧ 연간 마진 (DC24V 납품): "&amp;IF(ISNUMBER('마진 계산'!E17),TEXT('마진 계산'!E17,"#,##0")&amp;"원  (마진율 "&amp;TEXT('마진 계산'!F17,"0.0%")&amp;")","타겟 프라이스를 '마진 계산' 시트에 넣으면 여기에 표시됩니다")</f>
+        <v>⑧ 연간 마진 (DC24V 납품): 타겟 프라이스를 '마진 계산' 시트에 넣으면 여기에 표시됩니다</v>
+      </c>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A15:G15"/>
@@ -4700,6 +5469,7 @@
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A21:G21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4712,6 +5482,406 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <f aca="false">요약!C6</f>
+        <v>200</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <f aca="false">'프로젝트별 구성'!F9</f>
+        <v>392850</v>
+      </c>
+      <c r="E6" s="28"/>
+      <c r="F6" s="10" t="str">
+        <f aca="false">IF(E6="","",E6-D6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="29" t="str">
+        <f aca="false">IF(OR(E6="",E6=0),"",F6/E6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="9" t="str">
+        <f aca="false">IF(E6="","",C6*E6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="10" t="str">
+        <f aca="false">IF(E6="","",C6*F6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="33" t="n">
+        <f aca="false">요약!C6</f>
+        <v>200</v>
+      </c>
+      <c r="D7" s="34" t="n">
+        <f aca="false">'프로젝트별 구성'!F11</f>
+        <v>384750</v>
+      </c>
+      <c r="E7" s="35"/>
+      <c r="F7" s="36" t="str">
+        <f aca="false">IF(E7="","",E7-D7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="37" t="str">
+        <f aca="false">IF(OR(E7="",E7=0),"",F7/E7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="34" t="str">
+        <f aca="false">IF(E7="","",C7*E7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="36" t="str">
+        <f aca="false">IF(E7="","",C7*F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <f aca="false">요약!C7</f>
+        <v>300</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <f aca="false">'프로젝트별 구성'!F19</f>
+        <v>417600</v>
+      </c>
+      <c r="E8" s="28"/>
+      <c r="F8" s="10" t="str">
+        <f aca="false">IF(E8="","",E8-D8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="29" t="str">
+        <f aca="false">IF(OR(E8="",E8=0),"",F8/E8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="9" t="str">
+        <f aca="false">IF(E8="","",C8*E8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="10" t="str">
+        <f aca="false">IF(E8="","",C8*F8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <f aca="false">요약!C7</f>
+        <v>300</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <f aca="false">'프로젝트별 구성'!F21</f>
+        <v>406350</v>
+      </c>
+      <c r="E9" s="35"/>
+      <c r="F9" s="36" t="str">
+        <f aca="false">IF(E9="","",E9-D9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="37" t="str">
+        <f aca="false">IF(OR(E9="",E9=0),"",F9/E9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="34" t="str">
+        <f aca="false">IF(E9="","",C9*E9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="36" t="str">
+        <f aca="false">IF(E9="","",C9*F9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <f aca="false">요약!C8</f>
+        <v>50</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <f aca="false">'프로젝트별 구성'!F30</f>
+        <v>531250</v>
+      </c>
+      <c r="E10" s="28"/>
+      <c r="F10" s="10" t="str">
+        <f aca="false">IF(E10="","",E10-D10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="29" t="str">
+        <f aca="false">IF(OR(E10="",E10=0),"",F10/E10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="9" t="str">
+        <f aca="false">IF(E10="","",C10*E10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="10" t="str">
+        <f aca="false">IF(E10="","",C10*F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="33" t="n">
+        <f aca="false">요약!C8</f>
+        <v>50</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <f aca="false">'프로젝트별 구성'!F33</f>
+        <v>523150</v>
+      </c>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36" t="str">
+        <f aca="false">IF(E11="","",E11-D11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="37" t="str">
+        <f aca="false">IF(OR(E11="",E11=0),"",F11/E11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="34" t="str">
+        <f aca="false">IF(E11="","",C11*E11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="36" t="str">
+        <f aca="false">IF(E11="","",C11*F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="27" t="n">
+        <f aca="false">요약!C9</f>
+        <v>100</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <f aca="false">'프로젝트별 구성'!F44</f>
+        <v>1449500</v>
+      </c>
+      <c r="E12" s="28"/>
+      <c r="F12" s="10" t="str">
+        <f aca="false">IF(E12="","",E12-D12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="29" t="str">
+        <f aca="false">IF(OR(E12="",E12=0),"",F12/E12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="9" t="str">
+        <f aca="false">IF(E12="","",C12*E12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="10" t="str">
+        <f aca="false">IF(E12="","",C12*F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="39"/>
+      <c r="C17" s="9" t="n">
+        <f aca="false">C6*D6+C8*D8+C10*D10+C12*D12</f>
+        <v>375362500</v>
+      </c>
+      <c r="D17" s="9" t="str">
+        <f aca="false">IF((E6="")+(E8="")+(E10="")+(E12="")&gt;0,"타겟 "&amp;((E6="")+(E8="")+(E10="")+(E12=""))&amp;"건 미입력",H6+H8+H10+H12)</f>
+        <v>타겟 4건 미입력</v>
+      </c>
+      <c r="E17" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(D17),D17-C17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="41" t="str">
+        <f aca="false">IF(ISNUMBER(D17),E17/D17,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="39"/>
+      <c r="C18" s="9" t="n">
+        <f aca="false">C7*D7+C9*D9+C11*D11+C12*D12</f>
+        <v>369962500</v>
+      </c>
+      <c r="D18" s="9" t="str">
+        <f aca="false">IF((E7="")+(E9="")+(E11="")+(E12="")&gt;0,"타겟 "&amp;((E7="")+(E9="")+(E11="")+(E12=""))&amp;"건 미입력",H7+H9+H11+H12)</f>
+        <v>타겟 4건 미입력</v>
+      </c>
+      <c r="E18" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(D18),D18-C18,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="41" t="str">
+        <f aca="false">IF(ISNUMBER(D18),E18/D18,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="42" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="42" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F6:I12">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(ISNUMBER(F6),F6&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:F18">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(ISNUMBER(E17),E17&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -4729,55 +5899,55 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
-        <v>29</v>
+      <c r="A1" s="25" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>33</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="n">
+      <c r="A5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="27" t="s">
-        <v>40</v>
+      <c r="B5" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="44" t="s">
+        <v>60</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>886000</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="45" t="n">
         <v>0.45</v>
       </c>
       <c r="G5" s="10" t="n">
@@ -4786,22 +5956,22 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>42</v>
+      <c r="B6" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="44" t="s">
+        <v>62</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>873000</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="45" t="n">
         <v>0.45</v>
       </c>
       <c r="G6" s="10" t="n">
@@ -4810,22 +5980,22 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="n">
+      <c r="A7" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>45</v>
+      <c r="B7" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>65</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>855000</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="45" t="n">
         <v>0.45</v>
       </c>
       <c r="G7" s="10" t="n">
@@ -4834,22 +6004,22 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="27" t="s">
-        <v>47</v>
+      <c r="B8" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>67</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>928000</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="45" t="n">
         <v>0.45</v>
       </c>
       <c r="G8" s="10" t="n">
@@ -4858,22 +6028,22 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="n">
+      <c r="A9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>49</v>
+      <c r="B9" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>69</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>903000</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="45" t="n">
         <v>0.45</v>
       </c>
       <c r="G9" s="10" t="n">
@@ -4882,22 +6052,22 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>52</v>
+      <c r="B10" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>72</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>228000</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G10" s="10" t="n">
@@ -4906,22 +6076,22 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="n">
+      <c r="A11" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>54</v>
+      <c r="B11" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>74</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>202000</v>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G11" s="10" t="n">
@@ -4930,22 +6100,22 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="n">
+      <c r="A12" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>56</v>
+      <c r="B12" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>76</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>227000</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G12" s="10" t="n">
@@ -4954,22 +6124,22 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="n">
+      <c r="A13" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>58</v>
+      <c r="B13" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>78</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>227000</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G13" s="10" t="n">
@@ -4978,22 +6148,22 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="n">
+      <c r="A14" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>60</v>
+      <c r="B14" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>80</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>213000</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G14" s="10" t="n">
@@ -5002,22 +6172,22 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="n">
+      <c r="A15" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>62</v>
+      <c r="B15" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>82</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>161000</v>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G15" s="10" t="n">
@@ -5026,22 +6196,22 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="n">
+      <c r="A16" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>64</v>
+      <c r="B16" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>84</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>168000</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G16" s="10" t="n">
@@ -5050,22 +6220,22 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="n">
+      <c r="A17" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>66</v>
+      <c r="B17" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="46" t="s">
+        <v>86</v>
       </c>
       <c r="E17" s="9" t="n">
         <v>168000</v>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G17" s="10" t="n">
@@ -5074,22 +6244,22 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="n">
+      <c r="A18" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>68</v>
+      <c r="B18" s="43" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>88</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>311000</v>
       </c>
-      <c r="F18" s="28" t="n">
+      <c r="F18" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G18" s="10" t="n">
@@ -5098,22 +6268,22 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="n">
+      <c r="A19" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>70</v>
+      <c r="B19" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>90</v>
       </c>
       <c r="E19" s="9" t="n">
         <v>284000</v>
       </c>
-      <c r="F19" s="28" t="n">
+      <c r="F19" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G19" s="10" t="n">
@@ -5122,22 +6292,22 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="n">
+      <c r="A20" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="43" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>72</v>
+      <c r="D20" s="46" t="s">
+        <v>92</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>331000</v>
       </c>
-      <c r="F20" s="28" t="n">
+      <c r="F20" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G20" s="10" t="n">
@@ -5146,22 +6316,22 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="n">
+      <c r="A21" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>74</v>
+      <c r="B21" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>94</v>
       </c>
       <c r="E21" s="9" t="n">
         <v>346000</v>
       </c>
-      <c r="F21" s="28" t="n">
+      <c r="F21" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G21" s="10" t="n">
@@ -5170,22 +6340,22 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="n">
+      <c r="A22" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>76</v>
+      <c r="B22" s="43" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="46" t="s">
+        <v>96</v>
       </c>
       <c r="E22" s="9" t="n">
         <v>351000</v>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="45" t="n">
         <v>0.4</v>
       </c>
       <c r="G22" s="10" t="n">
@@ -5204,7 +6374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -5223,61 +6393,61 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="30" t="s">
-        <v>77</v>
+      <c r="A1" s="47" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="B3" s="32" t="n">
+      <c r="A3" s="48" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="49" t="n">
         <v>0.45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="32" t="n">
+      <c r="A4" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="49" t="n">
         <v>0.4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="H6" s="4" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>39</v>
+      <c r="A7" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>59</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">VLOOKUP(A7,단가표!$B$5:$G$22,4,FALSE())</f>
@@ -5291,11 +6461,11 @@
         <f aca="false">ROUND(C7*$B$4,0)</f>
         <v>349200</v>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F7" s="50" t="n">
         <f aca="false">D7-E7</f>
         <v>43650</v>
       </c>
-      <c r="G7" s="34" t="n">
+      <c r="G7" s="27" t="n">
         <f aca="false">요약!C6+요약!C8</f>
         <v>250</v>
       </c>
@@ -5303,16 +6473,16 @@
         <f aca="false">F7*G7</f>
         <v>10912500</v>
       </c>
-      <c r="I7" s="35" t="s">
-        <v>87</v>
+      <c r="I7" s="51" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>39</v>
+      <c r="A8" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>59</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">VLOOKUP(A8,단가표!$B$5:$G$22,4,FALSE())</f>
@@ -5326,11 +6496,11 @@
         <f aca="false">ROUND(C8*$B$4,0)</f>
         <v>371200</v>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F8" s="50" t="n">
         <f aca="false">D8-E8</f>
         <v>46400</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="27" t="n">
         <f aca="false">요약!C7</f>
         <v>300</v>
       </c>
@@ -5338,16 +6508,16 @@
         <f aca="false">F8*G8</f>
         <v>13920000</v>
       </c>
-      <c r="I8" s="35" t="s">
-        <v>88</v>
+      <c r="I8" s="51" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>39</v>
+      <c r="A9" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>59</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">VLOOKUP(A9,단가표!$B$5:$G$22,4,FALSE())</f>
@@ -5361,11 +6531,11 @@
         <f aca="false">ROUND(C9*$B$4,0)</f>
         <v>354400</v>
       </c>
-      <c r="F9" s="33" t="n">
+      <c r="F9" s="50" t="n">
         <f aca="false">D9-E9</f>
         <v>44300</v>
       </c>
-      <c r="G9" s="34" t="n">
+      <c r="G9" s="27" t="n">
         <f aca="false">요약!C9</f>
         <v>100</v>
       </c>
@@ -5373,16 +6543,16 @@
         <f aca="false">F9*G9</f>
         <v>4430000</v>
       </c>
-      <c r="I9" s="35" t="s">
+      <c r="I9" s="51" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>44</v>
+      <c r="A10" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>64</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">VLOOKUP(A10,단가표!$B$5:$G$22,4,FALSE())</f>
@@ -5396,11 +6566,11 @@
         <f aca="false">ROUND(C10*$B$4,0)</f>
         <v>342000</v>
       </c>
-      <c r="F10" s="33" t="n">
+      <c r="F10" s="50" t="n">
         <f aca="false">D10-E10</f>
         <v>42750</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="27" t="n">
         <f aca="false">요약!C6+요약!C8</f>
         <v>250</v>
       </c>
@@ -5408,16 +6578,16 @@
         <f aca="false">F10*G10</f>
         <v>10687500</v>
       </c>
-      <c r="I10" s="35" t="s">
-        <v>89</v>
+      <c r="I10" s="51" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>44</v>
+      <c r="A11" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>64</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">VLOOKUP(A11,단가표!$B$5:$G$22,4,FALSE())</f>
@@ -5431,11 +6601,11 @@
         <f aca="false">ROUND(C11*$B$4,0)</f>
         <v>361200</v>
       </c>
-      <c r="F11" s="33" t="n">
+      <c r="F11" s="50" t="n">
         <f aca="false">D11-E11</f>
         <v>45150</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="27" t="n">
         <f aca="false">요약!C7</f>
         <v>300</v>
       </c>
@@ -5443,43 +6613,43 @@
         <f aca="false">F11*G11</f>
         <v>13545000</v>
       </c>
-      <c r="I11" s="35" t="s">
-        <v>90</v>
+      <c r="I11" s="51" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
+      <c r="A13" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
       <c r="H13" s="16" t="n">
         <f aca="false">H7+H8+H9</f>
         <v>29262500</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
+      <c r="A14" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
       <c r="H14" s="16" t="n">
         <f aca="false">H9+H10+H11</f>
         <v>28662500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37" t="s">
-        <v>93</v>
+      <c r="A16" s="42" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -5497,7 +6667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -5513,81 +6683,81 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
-        <v>94</v>
+      <c r="A1" s="25" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="39" t="s">
+      <c r="A5" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
+      <c r="A6" s="48" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="41" t="str">
+      <c r="A8" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="55" t="str">
         <f aca="false">VLOOKUP(B8,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10)</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="9" t="n">
@@ -5600,30 +6770,30 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="43" t="n">
+      <c r="A9" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="57" t="n">
         <f aca="false">SUM(F8:F8)</f>
         <v>392850</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="41" t="str">
+      <c r="A10" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="55" t="str">
         <f aca="false">VLOOKUP(B10,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10 = 릴레이 6 + TR 4)</v>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="9" t="n">
@@ -5636,94 +6806,94 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="43" t="n">
+      <c r="A11" s="56" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="56"/>
+      <c r="C11" s="56"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="57" t="n">
         <f aca="false">SUM(F10:F10)</f>
         <v>384750</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>106</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
+      <c r="A12" s="58" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="58"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="39" t="s">
+      <c r="A15" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="53"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="53"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
+      <c r="A16" s="48" t="s">
+        <v>116</v>
+      </c>
+      <c r="B16" s="54" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="41" t="str">
+      <c r="A18" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="55" t="str">
         <f aca="false">VLOOKUP(B18,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 24 / 출력 16)</v>
       </c>
-      <c r="D18" s="25" t="n">
+      <c r="D18" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="9" t="n">
@@ -5736,30 +6906,30 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19" s="42"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="43" t="n">
+      <c r="A19" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" s="56"/>
+      <c r="C19" s="56"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="57" t="n">
         <f aca="false">SUM(F18:F18)</f>
         <v>417600</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="41" t="str">
+      <c r="A20" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="55" t="str">
         <f aca="false">VLOOKUP(B20,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 24 / 출력 16 = 릴레이 12 + TR 4)</v>
       </c>
-      <c r="D20" s="25" t="n">
+      <c r="D20" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="9" t="n">
@@ -5772,94 +6942,94 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="B21" s="42"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="43" t="n">
+      <c r="A21" s="56" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="56"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="57" t="n">
         <f aca="false">SUM(F20:F20)</f>
         <v>406350</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="45" t="s">
-        <v>108</v>
-      </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
+      <c r="A22" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="59"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38" t="s">
+      <c r="A24" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="B25" s="39" t="s">
+      <c r="A25" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="B26" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
+      <c r="A26" s="48" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
     </row>
     <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="41" t="str">
+      <c r="A28" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="55" t="str">
         <f aca="false">VLOOKUP(B28,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10)</v>
       </c>
-      <c r="D28" s="25" t="n">
+      <c r="D28" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="9" t="n">
@@ -5872,15 +7042,15 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25"/>
-      <c r="B29" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C29" s="41" t="str">
+      <c r="A29" s="26"/>
+      <c r="B29" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="55" t="str">
         <f aca="false">VLOOKUP(B29,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>아날로그 출력 2CH</v>
       </c>
-      <c r="D29" s="25" t="n">
+      <c r="D29" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="9" t="n">
@@ -5893,30 +7063,30 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="43" t="n">
+      <c r="A30" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="B30" s="56"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="57" t="n">
         <f aca="false">SUM(F28:F29)</f>
         <v>531250</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B31" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="41" t="str">
+      <c r="A31" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="55" t="str">
         <f aca="false">VLOOKUP(B31,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10 = 릴레이 6 + TR 4)</v>
       </c>
-      <c r="D31" s="25" t="n">
+      <c r="D31" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="9" t="n">
@@ -5929,15 +7099,15 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25"/>
-      <c r="B32" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C32" s="41" t="str">
+      <c r="A32" s="26"/>
+      <c r="B32" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="55" t="str">
         <f aca="false">VLOOKUP(B32,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>아날로그 출력 2CH</v>
       </c>
-      <c r="D32" s="25" t="n">
+      <c r="D32" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="9" t="n">
@@ -5950,94 +7120,94 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="43" t="n">
+      <c r="A33" s="56" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="56"/>
+      <c r="C33" s="56"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="57" t="n">
         <f aca="false">SUM(F31:F32)</f>
         <v>523150</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="B34" s="44"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="44"/>
-      <c r="E34" s="44"/>
-      <c r="F34" s="44"/>
+      <c r="A34" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="B34" s="58"/>
+      <c r="C34" s="58"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="58"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="38" t="s">
+      <c r="A36" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="52"/>
+      <c r="D36" s="52"/>
+      <c r="E36" s="52"/>
+      <c r="F36" s="52"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="B37" s="39" t="s">
+      <c r="A37" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="B38" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="C38" s="40"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
+      <c r="A38" s="48" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C38" s="54"/>
+      <c r="D38" s="54"/>
+      <c r="E38" s="54"/>
+      <c r="F38" s="54"/>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="B40" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" s="41" t="str">
+      <c r="A40" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B40" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="55" t="str">
         <f aca="false">VLOOKUP(B40,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>CPU + 이더넷 (입력 14 / 출력 10)</v>
       </c>
-      <c r="D40" s="25" t="n">
+      <c r="D40" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="9" t="n">
@@ -6050,15 +7220,15 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="25"/>
-      <c r="B41" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" s="41" t="str">
+      <c r="A41" s="26"/>
+      <c r="B41" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="C41" s="55" t="str">
         <f aca="false">VLOOKUP(B41,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>디지털 입력 16점</v>
       </c>
-      <c r="D41" s="25" t="n">
+      <c r="D41" s="26" t="n">
         <v>6</v>
       </c>
       <c r="E41" s="9" t="n">
@@ -6071,15 +7241,15 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="25"/>
-      <c r="B42" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" s="41" t="str">
+      <c r="A42" s="26"/>
+      <c r="B42" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" s="55" t="str">
         <f aca="false">VLOOKUP(B42,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>릴레이 출력 16점</v>
       </c>
-      <c r="D42" s="25" t="n">
+      <c r="D42" s="26" t="n">
         <v>4</v>
       </c>
       <c r="E42" s="9" t="n">
@@ -6092,15 +7262,15 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="25"/>
-      <c r="B43" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="C43" s="41" t="str">
+      <c r="A43" s="26"/>
+      <c r="B43" s="43" t="s">
+        <v>95</v>
+      </c>
+      <c r="C43" s="55" t="str">
         <f aca="false">VLOOKUP(B43,단가표!$B$5:$G$22,3,FALSE())</f>
         <v>아날로그 출력 4CH</v>
       </c>
-      <c r="D43" s="25" t="n">
+      <c r="D43" s="26" t="n">
         <v>1</v>
       </c>
       <c r="E43" s="9" t="n">
@@ -6113,27 +7283,27 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="42"/>
-      <c r="D44" s="42"/>
-      <c r="E44" s="42"/>
-      <c r="F44" s="43" t="n">
+      <c r="A44" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="B44" s="56"/>
+      <c r="C44" s="56"/>
+      <c r="D44" s="56"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="57" t="n">
         <f aca="false">SUM(F40:F43)</f>
         <v>1449500</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="45" t="s">
-        <v>113</v>
-      </c>
-      <c r="B45" s="45"/>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
+      <c r="A45" s="59" t="s">
+        <v>131</v>
+      </c>
+      <c r="B45" s="59"/>
+      <c r="C45" s="59"/>
+      <c r="D45" s="59"/>
+      <c r="E45" s="59"/>
+      <c r="F45" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="26">

</xml_diff>

<commit_message>
Mark MCC proposal as compliant per Techross confirmation (relay/TR either OK)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/PLC_견적_요약.xlsx
+++ b/PLC_견적_요약.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="253">
   <si>
     <r>
       <rPr>
@@ -606,7 +606,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">MCC — Techross </t>
+      <t xml:space="preserve">MCC — Schneider </t>
     </r>
     <r>
       <rPr>
@@ -616,7 +616,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">협의로 </t>
+      <t xml:space="preserve">제안이 </t>
     </r>
     <r>
       <rPr>
@@ -627,7 +627,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Schneider </t>
+      <t xml:space="preserve">Techross </t>
     </r>
     <r>
       <rPr>
@@ -637,7 +637,39 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">원안 확정</t>
+      <t xml:space="preserve">요구와 일치 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Techross </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -696,7 +728,26 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">40 TR / </t>
+      <t xml:space="preserve">40 (Relay·TR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무관</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) / </t>
     </r>
     <r>
       <rPr>
@@ -768,7 +819,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">② TSU · ANU · ANU-S: Schneider </t>
+      <t xml:space="preserve">② 4</t>
     </r>
     <r>
       <rPr>
@@ -777,7 +828,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">제안 구성 그대로 — </t>
+      <t xml:space="preserve">개 프로젝트 모두 </t>
     </r>
     <r>
       <rPr>
@@ -787,7 +838,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">RFQ </t>
+      <t xml:space="preserve">Schneider </t>
     </r>
     <r>
       <rPr>
@@ -796,7 +847,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">조건 충족</t>
+      <t xml:space="preserve">제안 구성이 </t>
     </r>
     <r>
       <rPr>
@@ -806,71 +857,147 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">Techross </t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">③ MCC: Schneider–Techross </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요구와 일치합니다 </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">협의로 원안</t>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(MCC</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(TM241CE40T </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">구성</t>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Relay·TR </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무관</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확정</t>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원안 점수 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Techross </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">③ MCC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 확장 모듈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개라 버스 확장 부품이 필요 없습니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
@@ -884,7 +1011,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">확장 모듈 </t>
+      <t xml:space="preserve">남은 보완은 서류</t>
     </r>
     <r>
       <rPr>
@@ -894,7 +1021,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">6</t>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
@@ -903,7 +1030,64 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">개라 버스 확장 부품은 필요 없습니다</t>
+      <t xml:space="preserve">제안 가격</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">외형도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CAD </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">등</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF375623"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뿐입니다</t>
     </r>
     <r>
       <rPr>
@@ -2716,7 +2900,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">·  MCC</t>
+      <t xml:space="preserve">·  4</t>
     </r>
     <r>
       <rPr>
@@ -2725,7 +2909,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">는 </t>
+      <t xml:space="preserve">개 프로젝트 모두 </t>
     </r>
     <r>
       <rPr>
@@ -2735,7 +2919,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Techross </t>
+      <t xml:space="preserve">Schneider </t>
     </r>
     <r>
       <rPr>
@@ -2744,7 +2928,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">협의로 </t>
+      <t xml:space="preserve">제안 구성 </t>
     </r>
     <r>
       <rPr>
@@ -2754,7 +2938,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Schneider </t>
+      <t xml:space="preserve">(Techross </t>
     </r>
     <r>
       <rPr>
@@ -2763,7 +2947,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">원안 확정</t>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -4090,29 +4284,208 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Relay Type Only (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공통사항 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5)</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">Relay·TR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무관 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Techross </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 2026-10-06)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">트랜지스터 출력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(TM241CE40T </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내장 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TR + TM3DQ16T + TM3DQ8T)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적합</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. RFQ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">문서의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'Relay Type Only'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Techross</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 무관하다고 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MCC I/O </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">점수</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">입력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">64 / </t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
@@ -4130,150 +4503,145 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">점 전부 트랜지스터 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(TM241CE40T </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">내장 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">TR + TM3DQ16T + TM3DQ8T)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">협의</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Schneider–Techross </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">협의로 원안</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(TR </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">출력</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확정 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(2026-10-06).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MCC I/O </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">점수</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">40 / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아날로그 출력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2CH (Techross </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">입력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">64 / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">출력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아날로그 출력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2CH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적합</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. RFQ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">문서의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
@@ -4291,157 +4659,45 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">입력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">102 / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">출력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">54 / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">아날로그 출력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4CH</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">입력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">64 / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">출력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">아날로그 출력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2CH</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Schneider–Techross </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">협의로 원안 점수 확정 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF1F3864"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(2026-10-06).</t>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대신 제안 점수가 맞다고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Techross </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>
@@ -7586,26 +7842,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">협의로 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Schneider </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원안 확정 </t>
+      <t xml:space="preserve">확인 </t>
     </r>
     <r>
       <rPr>
@@ -7653,7 +7890,26 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">40 (TR) / </t>
+      <t xml:space="preserve">40 (Relay·TR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무관</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) / </t>
     </r>
     <r>
       <rPr>
@@ -7691,7 +7947,16 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1CH</t>
+      <t xml:space="preserve">1CH — Schneider </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제안과 일치</t>
     </r>
   </si>
   <si>
@@ -9237,7 +9502,7 @@
     <numFmt numFmtId="169" formatCode="0.000"/>
     <numFmt numFmtId="170" formatCode="0.00"/>
   </numFmts>
-  <fonts count="61">
+  <fonts count="58">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9584,28 +9849,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF1F3864"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF1F3864"/>
-      <name val="맑은 고딕"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF1F3864"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF7F6000"/>
       <name val="맑은 고딕"/>
@@ -9785,7 +10028,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="90">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -10042,19 +10285,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="49" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="52" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="49" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10062,7 +10297,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="54" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="51" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10070,7 +10305,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="53" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10082,7 +10317,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="55" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="52" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10106,11 +10341,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="56" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="53" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10146,11 +10381,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="59" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="56" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="60" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="57" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10673,7 +10908,7 @@
       <c r="F18" s="22"/>
       <c r="G18" s="22"/>
     </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
         <v>25</v>
       </c>
@@ -10684,7 +10919,7 @@
       <c r="F19" s="23"/>
       <c r="G19" s="23"/>
     </row>
-    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
         <v>26</v>
       </c>
@@ -10754,8 +10989,8 @@
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="str">
-        <f aca="false">"⑨ Schneider 제안 검토: 반드시 수정 "&amp;COUNTIF('Schneider 제안 검토'!F7:F24,"✕")&amp;"건, 보완 "&amp;COUNTIF('Schneider 제안 검토'!F7:F24,"△")&amp;"건, Techross 협의 완료 "&amp;COUNTIF('Schneider 제안 검토'!F7:F24,"협의")&amp;"건  → 'Schneider 제안 검토' 시트"</f>
-        <v>⑨ Schneider 제안 검토: 반드시 수정 2건, 보완 5건, Techross 협의 완료 2건  → 'Schneider 제안 검토' 시트</v>
+        <f aca="false">"⑨ Schneider 제안 검토: 반드시 수정 "&amp;COUNTIF('Schneider 제안 검토'!F7:F24,"✕")&amp;"건, 보완 "&amp;COUNTIF('Schneider 제안 검토'!F7:F24,"△")&amp;"건  (구성은 4개 프로젝트 모두 적합)  → 'Schneider 제안 검토' 시트"</f>
+        <v>⑨ Schneider 제안 검토: 반드시 수정 2건, 보완 5건  (구성은 4개 프로젝트 모두 적합)  → 'Schneider 제안 검토' 시트</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -11998,8 +12233,8 @@
         <v>93</v>
       </c>
       <c r="E3" s="59" t="str">
-        <f aca="false">"✕ "&amp;COUNTIF(F7:F24,"✕")&amp;"건   △ "&amp;COUNTIF(F7:F24,"△")&amp;"건   ○ "&amp;COUNTIF(F7:F24,"○")&amp;"건   협의 완료 "&amp;COUNTIF(F7:F24,"협의")&amp;"건"</f>
-        <v>✕ 2건   △ 5건   ○ 9건   협의 완료 2건</v>
+        <f aca="false">"✕ "&amp;COUNTIF(F7:F24,"✕")&amp;"건   △ "&amp;COUNTIF(F7:F24,"△")&amp;"건   ○ "&amp;COUNTIF(F7:F24,"○")&amp;"건"</f>
+        <v>✕ 2건   △ 5건   ○ 11건</v>
       </c>
       <c r="F3" s="59"/>
       <c r="G3" s="59"/>
@@ -12096,7 +12331,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="n">
         <v>4</v>
       </c>
@@ -12112,11 +12347,11 @@
       <c r="E10" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="F10" s="64" t="s">
+      <c r="F10" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="G10" s="62" t="s">
         <v>117</v>
-      </c>
-      <c r="G10" s="65" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12127,19 +12362,19 @@
         <v>100</v>
       </c>
       <c r="C11" s="61" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="62" t="s">
+      <c r="E11" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="E11" s="62" t="s">
+      <c r="F11" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" s="62" t="s">
         <v>121</v>
-      </c>
-      <c r="F11" s="64" t="s">
-        <v>117</v>
-      </c>
-      <c r="G11" s="65" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12150,19 +12385,19 @@
         <v>100</v>
       </c>
       <c r="C12" s="61" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>125</v>
       </c>
       <c r="F12" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G12" s="62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12173,19 +12408,19 @@
         <v>100</v>
       </c>
       <c r="C13" s="61" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="62" t="s">
         <v>128</v>
-      </c>
-      <c r="E13" s="62" t="s">
-        <v>129</v>
       </c>
       <c r="F13" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12193,22 +12428,22 @@
         <v>8</v>
       </c>
       <c r="B14" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="64" t="s">
         <v>131</v>
       </c>
-      <c r="C14" s="66" t="s">
+      <c r="D14" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>133</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>134</v>
       </c>
       <c r="F14" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G14" s="62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12216,22 +12451,22 @@
         <v>9</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C15" s="61" t="s">
+        <v>134</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>137</v>
       </c>
       <c r="F15" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G15" s="62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12239,22 +12474,22 @@
         <v>10</v>
       </c>
       <c r="B16" s="60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C16" s="61" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>140</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>141</v>
       </c>
       <c r="F16" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12262,22 +12497,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C17" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="65" t="s">
         <v>145</v>
       </c>
-      <c r="F17" s="67" t="s">
+      <c r="G17" s="66" t="s">
         <v>146</v>
-      </c>
-      <c r="G17" s="68" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12285,22 +12520,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="66" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="64" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="F18" s="67" t="s">
         <v>150</v>
       </c>
-      <c r="F18" s="69" t="s">
+      <c r="G18" s="68" t="s">
         <v>151</v>
-      </c>
-      <c r="G18" s="70" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12308,22 +12543,22 @@
         <v>13</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C19" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="D19" s="62" t="s">
         <v>153</v>
       </c>
-      <c r="D19" s="62" t="s">
+      <c r="E19" s="62" t="s">
         <v>154</v>
       </c>
-      <c r="E19" s="62" t="s">
+      <c r="F19" s="65" t="s">
+        <v>145</v>
+      </c>
+      <c r="G19" s="69" t="s">
         <v>155</v>
-      </c>
-      <c r="F19" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="G19" s="71" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12331,22 +12566,22 @@
         <v>14</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>131</v>
-      </c>
-      <c r="C20" s="66" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="E20" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>159</v>
       </c>
       <c r="F20" s="63" t="s">
         <v>104</v>
       </c>
       <c r="G20" s="62" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12354,22 +12589,22 @@
         <v>15</v>
       </c>
       <c r="B21" s="60" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" s="64" t="s">
         <v>161</v>
       </c>
-      <c r="C21" s="66" t="s">
+      <c r="D21" s="62" t="s">
         <v>162</v>
       </c>
-      <c r="D21" s="62" t="s">
+      <c r="E21" s="62" t="s">
         <v>163</v>
       </c>
-      <c r="E21" s="62" t="s">
+      <c r="F21" s="65" t="s">
+        <v>145</v>
+      </c>
+      <c r="G21" s="69" t="s">
         <v>164</v>
-      </c>
-      <c r="F21" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="G21" s="71" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12377,22 +12612,22 @@
         <v>16</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C22" s="61" t="s">
+        <v>165</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="E22" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="E22" s="62" t="s">
+      <c r="F22" s="65" t="s">
+        <v>145</v>
+      </c>
+      <c r="G22" s="66" t="s">
         <v>168</v>
-      </c>
-      <c r="F22" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="G22" s="68" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12400,22 +12635,22 @@
         <v>17</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>161</v>
-      </c>
-      <c r="C23" s="66" t="s">
+        <v>160</v>
+      </c>
+      <c r="C23" s="64" t="s">
+        <v>169</v>
+      </c>
+      <c r="D23" s="62" t="s">
         <v>170</v>
       </c>
-      <c r="D23" s="62" t="s">
+      <c r="E23" s="62" t="s">
         <v>171</v>
       </c>
-      <c r="E23" s="62" t="s">
+      <c r="F23" s="67" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" s="70" t="s">
         <v>172</v>
-      </c>
-      <c r="F23" s="69" t="s">
-        <v>151</v>
-      </c>
-      <c r="G23" s="72" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12423,32 +12658,32 @@
         <v>18</v>
       </c>
       <c r="B24" s="60" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C24" s="61" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="62" t="s">
         <v>174</v>
       </c>
-      <c r="D24" s="62" t="s">
+      <c r="E24" s="62" t="s">
         <v>175</v>
       </c>
-      <c r="E24" s="62" t="s">
+      <c r="F24" s="65" t="s">
+        <v>145</v>
+      </c>
+      <c r="G24" s="69" t="s">
         <v>176</v>
       </c>
-      <c r="F24" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="G24" s="71" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="71" t="s">
         <v>177</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="73" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -12491,50 +12726,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="48" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="74" t="s">
+      <c r="A4" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B5" s="75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B5" s="73" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" s="74" t="s">
         <v>183</v>
       </c>
-      <c r="B6" s="76" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
@@ -12547,26 +12782,26 @@
         <v>66</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B8" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="77" t="str">
+      <c r="C8" s="75" t="str">
         <f aca="false">VLOOKUP(B8,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10)</v>
       </c>
@@ -12581,24 +12816,24 @@
         <f aca="false">D8*E8</f>
         <v>392850</v>
       </c>
-      <c r="G8" s="78" t="n">
+      <c r="G8" s="76" t="n">
         <f aca="false">D8*VLOOKUP(B8,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>873000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="79" t="s">
-        <v>190</v>
-      </c>
-      <c r="B9" s="79"/>
-      <c r="C9" s="79"/>
-      <c r="D9" s="79"/>
-      <c r="E9" s="79"/>
+      <c r="A9" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" s="77"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
       <c r="F9" s="54" t="n">
         <f aca="false">SUM(F8:F8)</f>
         <v>392850</v>
       </c>
-      <c r="G9" s="80" t="n">
+      <c r="G9" s="78" t="n">
         <f aca="false">SUM(G8:G8)</f>
         <v>873000</v>
       </c>
@@ -12610,7 +12845,7 @@
       <c r="B10" s="49" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="77" t="str">
+      <c r="C10" s="75" t="str">
         <f aca="false">VLOOKUP(B10,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10 = 릴레이 6 + TR 4)</v>
       </c>
@@ -12625,75 +12860,75 @@
         <f aca="false">D10*E10</f>
         <v>384750</v>
       </c>
-      <c r="G10" s="78" t="n">
+      <c r="G10" s="76" t="n">
         <f aca="false">D10*VLOOKUP(B10,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>855000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="79" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="79"/>
-      <c r="C11" s="79"/>
-      <c r="D11" s="79"/>
-      <c r="E11" s="79"/>
+      <c r="A11" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
       <c r="F11" s="54" t="n">
         <f aca="false">SUM(F10:F10)</f>
         <v>384750</v>
       </c>
-      <c r="G11" s="80" t="n">
+      <c r="G11" s="78" t="n">
         <f aca="false">SUM(G10:G10)</f>
         <v>855000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="81" t="s">
-        <v>192</v>
-      </c>
-      <c r="B12" s="81"/>
-      <c r="C12" s="81"/>
-      <c r="D12" s="81"/>
-      <c r="E12" s="81"/>
-      <c r="F12" s="81"/>
-      <c r="G12" s="81"/>
+      <c r="A12" s="79" t="s">
+        <v>191</v>
+      </c>
+      <c r="B12" s="79"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="79"/>
+      <c r="G12" s="79"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="74" t="s">
+      <c r="A14" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="74"/>
-      <c r="C14" s="74"/>
-      <c r="D14" s="74"/>
-      <c r="E14" s="74"/>
-      <c r="F14" s="74"/>
-      <c r="G14" s="74"/>
+      <c r="B14" s="72"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="72"/>
+      <c r="G14" s="72"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B15" s="75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B15" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="75"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="75"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="B16" s="76" t="s">
-        <v>193</v>
-      </c>
-      <c r="C16" s="76"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
+        <v>182</v>
+      </c>
+      <c r="B16" s="74" t="s">
+        <v>192</v>
+      </c>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
@@ -12706,26 +12941,26 @@
         <v>66</v>
       </c>
       <c r="D17" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B18" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="77" t="str">
+      <c r="C18" s="75" t="str">
         <f aca="false">VLOOKUP(B18,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 24 / 출력 16)</v>
       </c>
@@ -12740,24 +12975,24 @@
         <f aca="false">D18*E18</f>
         <v>417600</v>
       </c>
-      <c r="G18" s="78" t="n">
+      <c r="G18" s="76" t="n">
         <f aca="false">D18*VLOOKUP(B18,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>928000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="79" t="s">
-        <v>190</v>
-      </c>
-      <c r="B19" s="79"/>
-      <c r="C19" s="79"/>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
+      <c r="A19" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="B19" s="77"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
+      <c r="E19" s="77"/>
       <c r="F19" s="54" t="n">
         <f aca="false">SUM(F18:F18)</f>
         <v>417600</v>
       </c>
-      <c r="G19" s="80" t="n">
+      <c r="G19" s="78" t="n">
         <f aca="false">SUM(G18:G18)</f>
         <v>928000</v>
       </c>
@@ -12769,7 +13004,7 @@
       <c r="B20" s="49" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="77" t="str">
+      <c r="C20" s="75" t="str">
         <f aca="false">VLOOKUP(B20,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 24 / 출력 16 = 릴레이 12 + TR 4)</v>
       </c>
@@ -12784,75 +13019,75 @@
         <f aca="false">D20*E20</f>
         <v>406350</v>
       </c>
-      <c r="G20" s="78" t="n">
+      <c r="G20" s="76" t="n">
         <f aca="false">D20*VLOOKUP(B20,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>903000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="79" t="s">
-        <v>191</v>
-      </c>
-      <c r="B21" s="79"/>
-      <c r="C21" s="79"/>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
+      <c r="A21" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="77"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
       <c r="F21" s="54" t="n">
         <f aca="false">SUM(F20:F20)</f>
         <v>406350</v>
       </c>
-      <c r="G21" s="80" t="n">
+      <c r="G21" s="78" t="n">
         <f aca="false">SUM(G20:G20)</f>
         <v>903000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="82" t="s">
-        <v>194</v>
-      </c>
-      <c r="B22" s="82"/>
-      <c r="C22" s="82"/>
-      <c r="D22" s="82"/>
-      <c r="E22" s="82"/>
-      <c r="F22" s="82"/>
-      <c r="G22" s="82"/>
+      <c r="A22" s="80" t="s">
+        <v>193</v>
+      </c>
+      <c r="B22" s="80"/>
+      <c r="C22" s="80"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="80"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="74" t="s">
+      <c r="A24" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="74"/>
-      <c r="C24" s="74"/>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
+      <c r="B24" s="72"/>
+      <c r="C24" s="72"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="72"/>
+      <c r="F24" s="72"/>
+      <c r="G24" s="72"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B25" s="75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B25" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="75"/>
-      <c r="D25" s="75"/>
-      <c r="E25" s="75"/>
-      <c r="F25" s="75"/>
-      <c r="G25" s="75"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="B26" s="76" t="s">
-        <v>195</v>
-      </c>
-      <c r="C26" s="76"/>
-      <c r="D26" s="76"/>
-      <c r="E26" s="76"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="76"/>
+        <v>182</v>
+      </c>
+      <c r="B26" s="74" t="s">
+        <v>194</v>
+      </c>
+      <c r="C26" s="74"/>
+      <c r="D26" s="74"/>
+      <c r="E26" s="74"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="74"/>
     </row>
     <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
@@ -12865,26 +13100,26 @@
         <v>66</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B28" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="77" t="str">
+      <c r="C28" s="75" t="str">
         <f aca="false">VLOOKUP(B28,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10)</v>
       </c>
@@ -12899,7 +13134,7 @@
         <f aca="false">D28*E28</f>
         <v>392850</v>
       </c>
-      <c r="G28" s="78" t="n">
+      <c r="G28" s="76" t="n">
         <f aca="false">D28*VLOOKUP(B28,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>873000</v>
       </c>
@@ -12909,7 +13144,7 @@
       <c r="B29" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="77" t="str">
+      <c r="C29" s="75" t="str">
         <f aca="false">VLOOKUP(B29,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>아날로그 출력 2CH</v>
       </c>
@@ -12924,24 +13159,24 @@
         <f aca="false">D29*E29</f>
         <v>138400</v>
       </c>
-      <c r="G29" s="78" t="n">
+      <c r="G29" s="76" t="n">
         <f aca="false">D29*VLOOKUP(B29,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>346000</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="79" t="s">
-        <v>190</v>
-      </c>
-      <c r="B30" s="79"/>
-      <c r="C30" s="79"/>
-      <c r="D30" s="79"/>
-      <c r="E30" s="79"/>
+      <c r="A30" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="B30" s="77"/>
+      <c r="C30" s="77"/>
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
       <c r="F30" s="54" t="n">
         <f aca="false">SUM(F28:F29)</f>
         <v>531250</v>
       </c>
-      <c r="G30" s="80" t="n">
+      <c r="G30" s="78" t="n">
         <f aca="false">SUM(G28:G29)</f>
         <v>1219000</v>
       </c>
@@ -12953,7 +13188,7 @@
       <c r="B31" s="49" t="s">
         <v>75</v>
       </c>
-      <c r="C31" s="77" t="str">
+      <c r="C31" s="75" t="str">
         <f aca="false">VLOOKUP(B31,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU (입력 14 / 출력 10 = 릴레이 6 + TR 4)</v>
       </c>
@@ -12968,7 +13203,7 @@
         <f aca="false">D31*E31</f>
         <v>384750</v>
       </c>
-      <c r="G31" s="78" t="n">
+      <c r="G31" s="76" t="n">
         <f aca="false">D31*VLOOKUP(B31,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>855000</v>
       </c>
@@ -12978,7 +13213,7 @@
       <c r="B32" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="77" t="str">
+      <c r="C32" s="75" t="str">
         <f aca="false">VLOOKUP(B32,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>아날로그 출력 2CH</v>
       </c>
@@ -12993,75 +13228,75 @@
         <f aca="false">D32*E32</f>
         <v>138400</v>
       </c>
-      <c r="G32" s="78" t="n">
+      <c r="G32" s="76" t="n">
         <f aca="false">D32*VLOOKUP(B32,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>346000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="79" t="s">
-        <v>191</v>
-      </c>
-      <c r="B33" s="79"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="79"/>
-      <c r="E33" s="79"/>
+      <c r="A33" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" s="77"/>
+      <c r="C33" s="77"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
       <c r="F33" s="54" t="n">
         <f aca="false">SUM(F31:F32)</f>
         <v>523150</v>
       </c>
-      <c r="G33" s="80" t="n">
+      <c r="G33" s="78" t="n">
         <f aca="false">SUM(G31:G32)</f>
         <v>1201000</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="81" t="s">
-        <v>196</v>
-      </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
+      <c r="A34" s="79" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" s="79"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="79"/>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="79"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="74" t="s">
+      <c r="A36" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="74"/>
-      <c r="C36" s="74"/>
-      <c r="D36" s="74"/>
-      <c r="E36" s="74"/>
-      <c r="F36" s="74"/>
-      <c r="G36" s="74"/>
+      <c r="B36" s="72"/>
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
+      <c r="G36" s="72"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B37" s="75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="C37" s="75"/>
-      <c r="D37" s="75"/>
-      <c r="E37" s="75"/>
-      <c r="F37" s="75"/>
-      <c r="G37" s="75"/>
+      <c r="C37" s="73"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="73"/>
+      <c r="G37" s="73"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="B38" s="75" t="s">
-        <v>197</v>
-      </c>
-      <c r="C38" s="75"/>
-      <c r="D38" s="75"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="75"/>
+        <v>182</v>
+      </c>
+      <c r="B38" s="73" t="s">
+        <v>196</v>
+      </c>
+      <c r="C38" s="73"/>
+      <c r="D38" s="73"/>
+      <c r="E38" s="73"/>
+      <c r="F38" s="73"/>
+      <c r="G38" s="73"/>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
@@ -13074,26 +13309,26 @@
         <v>66</v>
       </c>
       <c r="D39" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="F39" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="G39" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B40" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="77" t="str">
+      <c r="C40" s="75" t="str">
         <f aca="false">VLOOKUP(B40,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>CPU + 이더넷 (입력 24 / 출력 16) — MCC, 견적에 없어 추정가</v>
       </c>
@@ -13108,7 +13343,7 @@
         <f aca="false">D40*E40</f>
         <v>423450</v>
       </c>
-      <c r="G40" s="78" t="n">
+      <c r="G40" s="76" t="n">
         <f aca="false">D40*VLOOKUP(B40,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>941000</v>
       </c>
@@ -13118,7 +13353,7 @@
       <c r="B41" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="77" t="str">
+      <c r="C41" s="75" t="str">
         <f aca="false">VLOOKUP(B41,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>디지털 입력 16점</v>
       </c>
@@ -13133,7 +13368,7 @@
         <f aca="false">D41*E41</f>
         <v>182400</v>
       </c>
-      <c r="G41" s="78" t="n">
+      <c r="G41" s="76" t="n">
         <f aca="false">D41*VLOOKUP(B41,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>456000</v>
       </c>
@@ -13143,7 +13378,7 @@
       <c r="B42" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="77" t="str">
+      <c r="C42" s="75" t="str">
         <f aca="false">VLOOKUP(B42,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>디지털 입력 8점</v>
       </c>
@@ -13158,7 +13393,7 @@
         <f aca="false">D42*E42</f>
         <v>80800</v>
       </c>
-      <c r="G42" s="78" t="n">
+      <c r="G42" s="76" t="n">
         <f aca="false">D42*VLOOKUP(B42,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>202000</v>
       </c>
@@ -13168,7 +13403,7 @@
       <c r="B43" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="C43" s="77" t="str">
+      <c r="C43" s="75" t="str">
         <f aca="false">VLOOKUP(B43,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>트랜지스터 출력 16점</v>
       </c>
@@ -13183,7 +13418,7 @@
         <f aca="false">D43*E43</f>
         <v>90800</v>
       </c>
-      <c r="G43" s="78" t="n">
+      <c r="G43" s="76" t="n">
         <f aca="false">D43*VLOOKUP(B43,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>227000</v>
       </c>
@@ -13193,7 +13428,7 @@
       <c r="B44" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="C44" s="77" t="str">
+      <c r="C44" s="75" t="str">
         <f aca="false">VLOOKUP(B44,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>트랜지스터 출력 8점</v>
       </c>
@@ -13208,7 +13443,7 @@
         <f aca="false">D44*E44</f>
         <v>67200</v>
       </c>
-      <c r="G44" s="78" t="n">
+      <c r="G44" s="76" t="n">
         <f aca="false">D44*VLOOKUP(B44,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>168000</v>
       </c>
@@ -13218,7 +13453,7 @@
       <c r="B45" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="C45" s="77" t="str">
+      <c r="C45" s="75" t="str">
         <f aca="false">VLOOKUP(B45,단가표!$B$5:$G$24,3,FALSE())</f>
         <v>아날로그 출력 2CH</v>
       </c>
@@ -13233,38 +13468,38 @@
         <f aca="false">D45*E45</f>
         <v>138400</v>
       </c>
-      <c r="G45" s="78" t="n">
+      <c r="G45" s="76" t="n">
         <f aca="false">D45*VLOOKUP(B45,단가표!$B$5:$G$24,4,FALSE())</f>
         <v>346000</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="79" t="s">
-        <v>190</v>
-      </c>
-      <c r="B46" s="79"/>
-      <c r="C46" s="79"/>
-      <c r="D46" s="79"/>
-      <c r="E46" s="79"/>
+      <c r="A46" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="77"/>
+      <c r="C46" s="77"/>
+      <c r="D46" s="77"/>
+      <c r="E46" s="77"/>
       <c r="F46" s="54" t="n">
         <f aca="false">SUM(F40:F45)</f>
         <v>983050</v>
       </c>
-      <c r="G46" s="80" t="n">
+      <c r="G46" s="78" t="n">
         <f aca="false">SUM(G40:G45)</f>
         <v>2340000</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="82" t="s">
-        <v>199</v>
-      </c>
-      <c r="B47" s="82"/>
-      <c r="C47" s="82"/>
-      <c r="D47" s="82"/>
-      <c r="E47" s="82"/>
-      <c r="F47" s="82"/>
-      <c r="G47" s="82"/>
+      <c r="A47" s="80" t="s">
+        <v>198</v>
+      </c>
+      <c r="B47" s="80"/>
+      <c r="C47" s="80"/>
+      <c r="D47" s="80"/>
+      <c r="E47" s="80"/>
+      <c r="F47" s="80"/>
+      <c r="G47" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -13325,52 +13560,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>201</v>
-      </c>
-      <c r="B3" s="83" t="n">
+        <v>200</v>
+      </c>
+      <c r="B3" s="81" t="n">
         <v>0.45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="81" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="B4" s="83" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>207</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>208</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13378,7 +13613,7 @@
         <v>73</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">VLOOKUP(A7,단가표!$B$5:$G$24,4,FALSE())</f>
@@ -13404,8 +13639,8 @@
         <f aca="false">F7*G7</f>
         <v>10912500</v>
       </c>
-      <c r="I7" s="84" t="s">
-        <v>211</v>
+      <c r="I7" s="82" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13413,7 +13648,7 @@
         <v>76</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">VLOOKUP(A8,단가표!$B$5:$G$24,4,FALSE())</f>
@@ -13439,8 +13674,8 @@
         <f aca="false">F8*G8</f>
         <v>13920000</v>
       </c>
-      <c r="I8" s="84" t="s">
-        <v>212</v>
+      <c r="I8" s="82" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13448,7 +13683,7 @@
         <v>78</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">VLOOKUP(A9,단가표!$B$5:$G$24,4,FALSE())</f>
@@ -13474,8 +13709,8 @@
         <f aca="false">F9*G9</f>
         <v>4705000</v>
       </c>
-      <c r="I9" s="84" t="s">
-        <v>213</v>
+      <c r="I9" s="82" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13483,7 +13718,7 @@
         <v>75</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">VLOOKUP(A10,단가표!$B$5:$G$24,4,FALSE())</f>
@@ -13509,8 +13744,8 @@
         <f aca="false">F10*G10</f>
         <v>10687500</v>
       </c>
-      <c r="I10" s="84" t="s">
-        <v>215</v>
+      <c r="I10" s="82" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13518,7 +13753,7 @@
         <v>77</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">VLOOKUP(A11,단가표!$B$5:$G$24,4,FALSE())</f>
@@ -13544,13 +13779,13 @@
         <f aca="false">F11*G11</f>
         <v>13545000</v>
       </c>
-      <c r="I11" s="84" t="s">
-        <v>216</v>
+      <c r="I11" s="82" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="42" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B13" s="42"/>
       <c r="C13" s="42"/>
@@ -13565,7 +13800,7 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="42" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B14" s="42"/>
       <c r="C14" s="42"/>
@@ -13580,7 +13815,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="46" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -13617,12 +13852,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="48" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13639,13 +13874,13 @@
         <v>66</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13653,18 +13888,18 @@
         <v>1</v>
       </c>
       <c r="B5" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" s="83" t="s">
         <v>223</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="D5" s="85" t="s">
-        <v>224</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>886000</v>
       </c>
-      <c r="F5" s="86" t="n">
+      <c r="F5" s="84" t="n">
         <v>0.45</v>
       </c>
       <c r="G5" s="10" t="n">
@@ -13680,15 +13915,15 @@
         <v>73</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="D6" s="85" t="s">
-        <v>225</v>
+        <v>209</v>
+      </c>
+      <c r="D6" s="83" t="s">
+        <v>224</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>873000</v>
       </c>
-      <c r="F6" s="86" t="n">
+      <c r="F6" s="84" t="n">
         <v>0.45</v>
       </c>
       <c r="G6" s="10" t="n">
@@ -13704,15 +13939,15 @@
         <v>75</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>214</v>
-      </c>
-      <c r="D7" s="85" t="s">
-        <v>226</v>
+        <v>213</v>
+      </c>
+      <c r="D7" s="83" t="s">
+        <v>225</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>855000</v>
       </c>
-      <c r="F7" s="86" t="n">
+      <c r="F7" s="84" t="n">
         <v>0.45</v>
       </c>
       <c r="G7" s="10" t="n">
@@ -13728,15 +13963,15 @@
         <v>76</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="D8" s="85" t="s">
-        <v>227</v>
+        <v>209</v>
+      </c>
+      <c r="D8" s="83" t="s">
+        <v>226</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>928000</v>
       </c>
-      <c r="F8" s="86" t="n">
+      <c r="F8" s="84" t="n">
         <v>0.45</v>
       </c>
       <c r="G8" s="10" t="n">
@@ -13752,15 +13987,15 @@
         <v>77</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>214</v>
-      </c>
-      <c r="D9" s="85" t="s">
-        <v>228</v>
+        <v>213</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>227</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>903000</v>
       </c>
-      <c r="F9" s="86" t="n">
+      <c r="F9" s="84" t="n">
         <v>0.45</v>
       </c>
       <c r="G9" s="10" t="n">
@@ -13776,15 +14011,15 @@
         <v>80</v>
       </c>
       <c r="C10" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D10" s="85" t="s">
         <v>229</v>
-      </c>
-      <c r="D10" s="87" t="s">
-        <v>230</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>228000</v>
       </c>
-      <c r="F10" s="86" t="n">
+      <c r="F10" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G10" s="10" t="n">
@@ -13800,15 +14035,15 @@
         <v>82</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D11" s="87" t="s">
-        <v>231</v>
+        <v>228</v>
+      </c>
+      <c r="D11" s="85" t="s">
+        <v>230</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>202000</v>
       </c>
-      <c r="F11" s="86" t="n">
+      <c r="F11" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G11" s="10" t="n">
@@ -13821,18 +14056,18 @@
         <v>8</v>
       </c>
       <c r="B12" s="49" t="s">
+        <v>231</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="85" t="s">
         <v>232</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D12" s="87" t="s">
-        <v>233</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>227000</v>
       </c>
-      <c r="F12" s="86" t="n">
+      <c r="F12" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G12" s="10" t="n">
@@ -13848,15 +14083,15 @@
         <v>83</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D13" s="87" t="s">
-        <v>234</v>
+        <v>228</v>
+      </c>
+      <c r="D13" s="85" t="s">
+        <v>233</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>227000</v>
       </c>
-      <c r="F13" s="86" t="n">
+      <c r="F13" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G13" s="10" t="n">
@@ -13869,18 +14104,18 @@
         <v>10</v>
       </c>
       <c r="B14" s="49" t="s">
+        <v>234</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="85" t="s">
         <v>235</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D14" s="87" t="s">
-        <v>236</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>213000</v>
       </c>
-      <c r="F14" s="86" t="n">
+      <c r="F14" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G14" s="10" t="n">
@@ -13893,18 +14128,18 @@
         <v>11</v>
       </c>
       <c r="B15" s="49" t="s">
+        <v>236</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="85" t="s">
         <v>237</v>
-      </c>
-      <c r="C15" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D15" s="87" t="s">
-        <v>238</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>161000</v>
       </c>
-      <c r="F15" s="86" t="n">
+      <c r="F15" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G15" s="10" t="n">
@@ -13920,15 +14155,15 @@
         <v>84</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D16" s="87" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="D16" s="85" t="s">
+        <v>238</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>168000</v>
       </c>
-      <c r="F16" s="86" t="n">
+      <c r="F16" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G16" s="10" t="n">
@@ -13941,18 +14176,18 @@
         <v>13</v>
       </c>
       <c r="B17" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D17" s="85" t="s">
         <v>240</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D17" s="87" t="s">
-        <v>241</v>
       </c>
       <c r="E17" s="9" t="n">
         <v>168000</v>
       </c>
-      <c r="F17" s="86" t="n">
+      <c r="F17" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G17" s="10" t="n">
@@ -13965,18 +14200,18 @@
         <v>14</v>
       </c>
       <c r="B18" s="49" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D18" s="85" t="s">
         <v>242</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D18" s="87" t="s">
-        <v>243</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>311000</v>
       </c>
-      <c r="F18" s="86" t="n">
+      <c r="F18" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G18" s="10" t="n">
@@ -13989,18 +14224,18 @@
         <v>15</v>
       </c>
       <c r="B19" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D19" s="85" t="s">
         <v>244</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D19" s="87" t="s">
-        <v>245</v>
       </c>
       <c r="E19" s="9" t="n">
         <v>284000</v>
       </c>
-      <c r="F19" s="86" t="n">
+      <c r="F19" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G19" s="10" t="n">
@@ -14013,18 +14248,18 @@
         <v>16</v>
       </c>
       <c r="B20" s="49" t="s">
+        <v>245</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D20" s="85" t="s">
         <v>246</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D20" s="87" t="s">
-        <v>247</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>331000</v>
       </c>
-      <c r="F20" s="86" t="n">
+      <c r="F20" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G20" s="10" t="n">
@@ -14040,15 +14275,15 @@
         <v>85</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D21" s="87" t="s">
-        <v>248</v>
+        <v>228</v>
+      </c>
+      <c r="D21" s="85" t="s">
+        <v>247</v>
       </c>
       <c r="E21" s="9" t="n">
         <v>346000</v>
       </c>
-      <c r="F21" s="86" t="n">
+      <c r="F21" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G21" s="10" t="n">
@@ -14061,18 +14296,18 @@
         <v>18</v>
       </c>
       <c r="B22" s="49" t="s">
+        <v>248</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="D22" s="85" t="s">
         <v>249</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D22" s="87" t="s">
-        <v>250</v>
       </c>
       <c r="E22" s="9" t="n">
         <v>351000</v>
       </c>
-      <c r="F22" s="86" t="n">
+      <c r="F22" s="84" t="n">
         <v>0.4</v>
       </c>
       <c r="G22" s="10" t="n">
@@ -14081,33 +14316,33 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="88" t="s">
-        <v>251</v>
-      </c>
-      <c r="B23" s="88"/>
-      <c r="C23" s="88"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="88"/>
+      <c r="A23" s="86" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="86"/>
+      <c r="G23" s="86"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B24" s="49" t="s">
         <v>78</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="D24" s="89" t="s">
-        <v>252</v>
-      </c>
-      <c r="E24" s="90" t="n">
+        <v>209</v>
+      </c>
+      <c r="D24" s="87" t="s">
+        <v>251</v>
+      </c>
+      <c r="E24" s="88" t="n">
         <v>941000</v>
       </c>
-      <c r="F24" s="91" t="n">
+      <c r="F24" s="89" t="n">
         <v>0.45</v>
       </c>
       <c r="G24" s="10" t="n">
@@ -14117,7 +14352,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Techross quotation (DC/AC) and internal margin summary; MCC price 1,170,000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/PLC_견적_요약.xlsx
+++ b/PLC_견적_요약.xlsx
@@ -4065,7 +4065,7 @@
     <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="26" t="str">
         <f aca="false">"⑧ LS 타겟 기준 연간 마진 (DC24V): "&amp;IF(ISNUMBER('마진 계산'!E30),TEXT('마진 계산'!E30,"#,##0")&amp;"원 (마진율 "&amp;TEXT('마진 계산'!F30,"0.0%")&amp;")  /  희망 마진("&amp;TEXT('마진 계산'!B4,"0%")&amp;")까지 연간 추가 특가 "&amp;TEXT('마진 계산'!G30,"#,##0")&amp;"원 (프로젝트별로 각각 맞출 때)  — 묶음 전체로는 "&amp;IF('마진 계산'!F30&gt;='마진 계산'!B4,"추가 특가 없이 달성","추가 특가 필요"),"LS 타겟 프라이스를 '마진 계산' 시트에 넣으면 여기에 표시됩니다")</f>
-        <v>⑧ LS 타겟 기준 연간 마진 (DC24V): 117,495,000원 (마진율 26.4%)  /  희망 마진(20%)까지 연간 추가 특가 26,690,000원 (프로젝트별로 각각 맞출 때)  — 묶음 전체로는 추가 특가 없이 달성</v>
+        <v>⑧ LS 타겟 기준 연간 마진 (DC24V): 114,495,000원 (마진율 25.9%)  /  희망 마진(20%)까지 연간 추가 특가 29,090,000원 (프로젝트별로 각각 맞출 때)  — 묶음 전체로는 추가 특가 없이 달성</v>
       </c>
       <c r="B28" s="26"/>
       <c r="C28" s="26"/>
@@ -4077,7 +4077,7 @@
     <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="str">
         <f aca="false">IF(NOT(ISNUMBER('마진 계산'!F14)),"⑨ MCC 마진: LS 타겟을 넣으면 표시됩니다",IF('마진 계산'!F14&lt;0,"⑨ MCC는 LS 타겟 대비 1대 "&amp;TEXT('마진 계산'!F14,"#,##0")&amp;"원 ("&amp;TEXT('마진 계산'!G14,"0.0%")&amp;"), 연 "&amp;TEXT('마진 계산'!I14,"#,##0")&amp;"원 손실 → 묶음 전체 마진("&amp;TEXT('마진 계산'!F30,"0.0%")&amp;")으로 흡수","⑨ MCC 마진: 1대 "&amp;TEXT('마진 계산'!F14,"#,##0")&amp;"원 ("&amp;TEXT('마진 계산'!G14,"0.0%")&amp;")"))</f>
-        <v>⑨ MCC는 LS 타겟 대비 1대 -26,900원 (-2.2%), 연 -2,690,000원 손실 → 묶음 전체 마진(26.4%)으로 흡수</v>
+        <v>⑨ MCC는 LS 타겟 대비 1대 -56,900원 (-4.9%), 연 -5,690,000원 손실 → 묶음 전체 마진(25.9%)으로 흡수</v>
       </c>
       <c r="B29" s="27"/>
       <c r="C29" s="27"/>
@@ -4424,7 +4424,7 @@
         <v>100</v>
       </c>
       <c r="D14" s="35" t="n">
-        <v>1200000</v>
+        <v>1170000</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">'프로젝트별 구성'!F47</f>
@@ -4432,19 +4432,19 @@
       </c>
       <c r="F14" s="36" t="n">
         <f aca="false">IF(D14="","",D14-E14)</f>
-        <v>-26900</v>
+        <v>-56900</v>
       </c>
       <c r="G14" s="37" t="n">
         <f aca="false">IF(OR(D14="",D14=0),"",F14/D14)</f>
-        <v>-0.0224166666666667</v>
+        <v>-0.0486324786324786</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">IF(D14="","",C14*D14)</f>
-        <v>120000000</v>
+        <v>117000000</v>
       </c>
       <c r="I14" s="36" t="n">
         <f aca="false">IF(D14="","",C14*F14)</f>
-        <v>-2690000</v>
+        <v>-5690000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="C25" s="10" t="n">
         <f aca="false">IF(D14="","",ROUND(D14*(1-$B$4),0))</f>
-        <v>960000</v>
+        <v>936000</v>
       </c>
       <c r="D25" s="10" t="n">
         <f aca="false">E14</f>
@@ -4745,11 +4745,11 @@
       </c>
       <c r="E25" s="42" t="n">
         <f aca="false">IF(C25="","",MAX(D25-C25,0))</f>
-        <v>266900</v>
+        <v>290900</v>
       </c>
       <c r="F25" s="43" t="n">
         <f aca="false">IF(C25="","",E25/D25)</f>
-        <v>0.217540141820849</v>
+        <v>0.237101638275328</v>
       </c>
       <c r="G25" s="44" t="n">
         <f aca="false">IFERROR(D25/'프로젝트별 구성'!G47,"")</f>
@@ -4757,11 +4757,11 @@
       </c>
       <c r="H25" s="45" t="n">
         <f aca="false">IF(C25="","",IFERROR(MIN(C25,D25)/'프로젝트별 구성'!G47,""))</f>
-        <v>0.28452874925904</v>
+        <v>0.277415530527564</v>
       </c>
       <c r="I25" s="11" t="n">
         <f aca="false">IF(C25="","",E25*C14)</f>
-        <v>26690000</v>
+        <v>29090000</v>
       </c>
       <c r="J25" s="46" t="str">
         <f aca="false">IF(C25="","타겟 입력 전",IF(E25=0,"OK — 지금 단가로 희망 마진 확보","추가 특가 필요"))</f>
@@ -4810,19 +4810,19 @@
       </c>
       <c r="D30" s="10" t="n">
         <f aca="false">IF((D8="")+(D10="")+(D12="")+(D14="")&gt;0,"타겟 "&amp;((D8="")+(D10="")+(D12="")+(D14=""))&amp;"건 미입력",H8+H10+H12+H14)</f>
-        <v>444900000</v>
+        <v>441900000</v>
       </c>
       <c r="E30" s="49" t="n">
         <f aca="false">IF(ISNUMBER(D30),D30-C30,"")</f>
-        <v>117495000</v>
+        <v>114495000</v>
       </c>
       <c r="F30" s="50" t="n">
         <f aca="false">IF(ISNUMBER(D30),E30/D30,"")</f>
-        <v>0.264093054619016</v>
+        <v>0.259097080787509</v>
       </c>
       <c r="G30" s="51" t="n">
         <f aca="false">IF(ISNUMBER(D30),I19+I21+I23+I25,"")</f>
-        <v>26690000</v>
+        <v>29090000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4836,19 +4836,19 @@
       </c>
       <c r="D31" s="10" t="n">
         <f aca="false">IF((D9="")+(D11="")+(D13="")+(D14="")&gt;0,"타겟 "&amp;((D9="")+(D11="")+(D13="")+(D14=""))&amp;"건 미입력",H9+H11+H13+H14)</f>
-        <v>444900000</v>
+        <v>441900000</v>
       </c>
       <c r="E31" s="49" t="n">
         <f aca="false">IF(ISNUMBER(D31),D31-C31,"")</f>
-        <v>122295000</v>
+        <v>119295000</v>
       </c>
       <c r="F31" s="50" t="n">
         <f aca="false">IF(ISNUMBER(D31),E31/D31,"")</f>
-        <v>0.274881995954147</v>
+        <v>0.269959266802444</v>
       </c>
       <c r="G31" s="51" t="n">
         <f aca="false">IF(ISNUMBER(D31),I20+I22+I24+I25,"")</f>
-        <v>26690000</v>
+        <v>29090000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>